<commit_message>
Add split_regions: auto-decompose bbox into obstacle-free rectangles
When bbox_from selects an L-shaped, U-shaped, or other non-rectangular
group of geometry items, the single rectangular region would also cover
non-selected items within its bounding box. With split_regions enabled,
the tool recursively splits along x/y/z axes to create the minimum
number of rectangular regions that avoid all non-selected items.

- Add _item_overlaps_bbox and _decompose_selected_items functions
- Add split_regions option in JSON bbox_from config
- Add split_regions column in Excel regions sheet
- Update template with split_regions example
- Update docs with usage examples and algorithm description

Generated with [Claude Code](https://claude.ai/code)
via [Happy](https://happy.engineering)

Co-Authored-By: Claude <noreply@anthropic.com>
Co-Authored-By: Happy <yesreply@happy.engineering>
</commit_message>
<xml_diff>
--- a/examples/FloXML/Spreadsheets/volume_regions_template.xlsx
+++ b/examples/FloXML/Spreadsheets/volume_regions_template.xlsx
@@ -631,7 +631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T3"/>
+  <dimension ref="A1:U4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -654,6 +654,7 @@
     <col width="18" customWidth="1" min="18" max="18"/>
     <col width="18" customWidth="1" min="19" max="19"/>
     <col width="18" customWidth="1" min="20" max="20"/>
+    <col width="18" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -724,35 +725,40 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
+          <t>split_regions</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
           <t>active</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>hidden</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>localized_grid</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>x_grid_constraint</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>y_grid_constraint</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>z_grid_constraint</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>all_grid_constraint</t>
         </is>
@@ -844,15 +850,62 @@
       </c>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr">
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr">
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Grid Constraint 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Split Region L-Shape</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>C1,C2,C3,C4,C7</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>0.05</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr">
         <is>
           <t>Grid Constraint 1</t>
         </is>

</xml_diff>